<commit_message>
fix row formatting in excel
</commit_message>
<xml_diff>
--- a/SMAEndpointDirectory.xlsx
+++ b/SMAEndpointDirectory.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\smahoney\Documents\GitHub\SMA-Endpoint-Directory\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91425C0F-03BE-422F-8C29-BCC2160E9835}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFCB33D1-365F-43E4-90F2-EAE2EC212DBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{CA3CA786-33B6-407A-829D-32600277E3D1}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{CA3CA786-33B6-407A-829D-32600277E3D1}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="8" r:id="rId1"/>
@@ -2914,7 +2914,7 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="239">
+  <cellXfs count="225">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -3418,6 +3418,152 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="8" borderId="1" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="5" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="5" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="14" borderId="13" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="3" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -3426,194 +3572,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="12" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="3" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="8" borderId="1" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="5" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="5" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="11" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="11" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="10" borderId="1" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="14" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="14" borderId="13" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="10">
     <cellStyle name="20% - Accent4" xfId="1" builtinId="42"/>
@@ -3955,40 +3913,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="23.7" customHeight="1">
-      <c r="A1" s="187" t="s">
+      <c r="A1" s="202" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="187"/>
-      <c r="C1" s="187"/>
-      <c r="D1" s="187"/>
-      <c r="E1" s="187"/>
-      <c r="F1" s="187"/>
-      <c r="G1" s="187"/>
-      <c r="H1" s="187"/>
-      <c r="I1" s="187"/>
-      <c r="J1" s="187"/>
-      <c r="K1" s="187"/>
-      <c r="L1" s="187"/>
-      <c r="M1" s="187"/>
+      <c r="B1" s="202"/>
+      <c r="C1" s="202"/>
+      <c r="D1" s="202"/>
+      <c r="E1" s="202"/>
+      <c r="F1" s="202"/>
+      <c r="G1" s="202"/>
+      <c r="H1" s="202"/>
+      <c r="I1" s="202"/>
+      <c r="J1" s="202"/>
+      <c r="K1" s="202"/>
+      <c r="L1" s="202"/>
+      <c r="M1" s="202"/>
     </row>
     <row r="3" spans="1:13" ht="121.2" customHeight="1">
       <c r="A3" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="194" t="s">
+      <c r="B3" s="209" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="195"/>
-      <c r="D3" s="195"/>
-      <c r="E3" s="195"/>
-      <c r="F3" s="195"/>
-      <c r="G3" s="195"/>
-      <c r="H3" s="195"/>
-      <c r="I3" s="195"/>
-      <c r="J3" s="195"/>
-      <c r="K3" s="195"/>
-      <c r="L3" s="195"/>
-      <c r="M3" s="195"/>
+      <c r="C3" s="210"/>
+      <c r="D3" s="210"/>
+      <c r="E3" s="210"/>
+      <c r="F3" s="210"/>
+      <c r="G3" s="210"/>
+      <c r="H3" s="210"/>
+      <c r="I3" s="210"/>
+      <c r="J3" s="210"/>
+      <c r="K3" s="210"/>
+      <c r="L3" s="210"/>
+      <c r="M3" s="210"/>
     </row>
     <row r="5" spans="1:13" ht="11.7" customHeight="1">
       <c r="A5" s="16"/>
@@ -4006,41 +3964,41 @@
       <c r="M5" s="17"/>
     </row>
     <row r="6" spans="1:13" ht="13.95" customHeight="1">
-      <c r="A6" s="204" t="s">
+      <c r="A6" s="219" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="205"/>
-      <c r="C6" s="205"/>
-      <c r="D6" s="205"/>
-      <c r="E6" s="205"/>
-      <c r="F6" s="205"/>
-      <c r="G6" s="205"/>
-      <c r="H6" s="205"/>
-      <c r="I6" s="205"/>
-      <c r="J6" s="205"/>
-      <c r="K6" s="205"/>
-      <c r="L6" s="205"/>
-      <c r="M6" s="205"/>
+      <c r="B6" s="220"/>
+      <c r="C6" s="220"/>
+      <c r="D6" s="220"/>
+      <c r="E6" s="220"/>
+      <c r="F6" s="220"/>
+      <c r="G6" s="220"/>
+      <c r="H6" s="220"/>
+      <c r="I6" s="220"/>
+      <c r="J6" s="220"/>
+      <c r="K6" s="220"/>
+      <c r="L6" s="220"/>
+      <c r="M6" s="220"/>
     </row>
     <row r="7" spans="1:13" ht="13.95" customHeight="1">
       <c r="A7" s="9"/>
     </row>
     <row r="8" spans="1:13" ht="13.95" customHeight="1">
-      <c r="A8" s="197" t="s">
+      <c r="A8" s="212" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="197"/>
-      <c r="C8" s="197"/>
-      <c r="D8" s="197"/>
-      <c r="E8" s="197"/>
-      <c r="F8" s="197"/>
-      <c r="G8" s="197"/>
-      <c r="H8" s="197"/>
-      <c r="I8" s="197"/>
-      <c r="J8" s="197"/>
-      <c r="K8" s="197"/>
-      <c r="L8" s="197"/>
-      <c r="M8" s="197"/>
+      <c r="B8" s="212"/>
+      <c r="C8" s="212"/>
+      <c r="D8" s="212"/>
+      <c r="E8" s="212"/>
+      <c r="F8" s="212"/>
+      <c r="G8" s="212"/>
+      <c r="H8" s="212"/>
+      <c r="I8" s="212"/>
+      <c r="J8" s="212"/>
+      <c r="K8" s="212"/>
+      <c r="L8" s="212"/>
+      <c r="M8" s="212"/>
     </row>
     <row r="9" spans="1:13" ht="27.45" customHeight="1">
       <c r="A9" s="150" t="s">
@@ -4052,21 +4010,21 @@
       <c r="C9" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D9" s="188" t="s">
+      <c r="D9" s="203" t="s">
         <v>8</v>
       </c>
-      <c r="E9" s="189"/>
-      <c r="F9" s="189"/>
-      <c r="G9" s="189"/>
-      <c r="H9" s="189"/>
-      <c r="I9" s="189"/>
-      <c r="J9" s="189"/>
-      <c r="K9" s="189"/>
-      <c r="L9" s="189"/>
-      <c r="M9" s="189"/>
+      <c r="E9" s="204"/>
+      <c r="F9" s="204"/>
+      <c r="G9" s="204"/>
+      <c r="H9" s="204"/>
+      <c r="I9" s="204"/>
+      <c r="J9" s="204"/>
+      <c r="K9" s="204"/>
+      <c r="L9" s="204"/>
+      <c r="M9" s="204"/>
     </row>
     <row r="10" spans="1:13">
-      <c r="A10" s="192" t="s">
+      <c r="A10" s="207" t="s">
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
@@ -4075,126 +4033,126 @@
       <c r="C10" s="152" t="s">
         <v>11</v>
       </c>
-      <c r="D10" s="196" t="s">
+      <c r="D10" s="211" t="s">
         <v>12</v>
       </c>
-      <c r="E10" s="196"/>
-      <c r="F10" s="196"/>
-      <c r="G10" s="196"/>
-      <c r="H10" s="196"/>
-      <c r="I10" s="196"/>
-      <c r="J10" s="196"/>
-      <c r="K10" s="196"/>
-      <c r="L10" s="196"/>
-      <c r="M10" s="196"/>
+      <c r="E10" s="211"/>
+      <c r="F10" s="211"/>
+      <c r="G10" s="211"/>
+      <c r="H10" s="211"/>
+      <c r="I10" s="211"/>
+      <c r="J10" s="211"/>
+      <c r="K10" s="211"/>
+      <c r="L10" s="211"/>
+      <c r="M10" s="211"/>
     </row>
     <row r="11" spans="1:13" ht="31.2" customHeight="1">
-      <c r="A11" s="193"/>
+      <c r="A11" s="208"/>
       <c r="B11" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C11" s="153" t="s">
         <v>11</v>
       </c>
-      <c r="D11" s="175" t="s">
+      <c r="D11" s="190" t="s">
         <v>14</v>
       </c>
-      <c r="E11" s="175"/>
-      <c r="F11" s="175"/>
-      <c r="G11" s="175"/>
-      <c r="H11" s="175"/>
-      <c r="I11" s="175"/>
-      <c r="J11" s="175"/>
-      <c r="K11" s="175"/>
-      <c r="L11" s="175"/>
-      <c r="M11" s="175"/>
+      <c r="E11" s="190"/>
+      <c r="F11" s="190"/>
+      <c r="G11" s="190"/>
+      <c r="H11" s="190"/>
+      <c r="I11" s="190"/>
+      <c r="J11" s="190"/>
+      <c r="K11" s="190"/>
+      <c r="L11" s="190"/>
+      <c r="M11" s="190"/>
     </row>
     <row r="12" spans="1:13" ht="22.2" customHeight="1">
-      <c r="A12" s="193"/>
+      <c r="A12" s="208"/>
       <c r="B12" s="2" t="s">
         <v>15</v>
       </c>
       <c r="C12" s="153" t="s">
         <v>11</v>
       </c>
-      <c r="D12" s="175" t="s">
+      <c r="D12" s="190" t="s">
         <v>16</v>
       </c>
-      <c r="E12" s="175"/>
-      <c r="F12" s="175"/>
-      <c r="G12" s="175"/>
-      <c r="H12" s="175"/>
-      <c r="I12" s="175"/>
-      <c r="J12" s="175"/>
-      <c r="K12" s="175"/>
-      <c r="L12" s="175"/>
-      <c r="M12" s="175"/>
+      <c r="E12" s="190"/>
+      <c r="F12" s="190"/>
+      <c r="G12" s="190"/>
+      <c r="H12" s="190"/>
+      <c r="I12" s="190"/>
+      <c r="J12" s="190"/>
+      <c r="K12" s="190"/>
+      <c r="L12" s="190"/>
+      <c r="M12" s="190"/>
     </row>
     <row r="13" spans="1:13" ht="39.450000000000003" customHeight="1">
-      <c r="A13" s="193"/>
+      <c r="A13" s="208"/>
       <c r="B13" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C13" s="153" t="s">
         <v>11</v>
       </c>
-      <c r="D13" s="175" t="s">
+      <c r="D13" s="190" t="s">
         <v>18</v>
       </c>
-      <c r="E13" s="175"/>
-      <c r="F13" s="175"/>
-      <c r="G13" s="175"/>
-      <c r="H13" s="175"/>
-      <c r="I13" s="175"/>
-      <c r="J13" s="175"/>
-      <c r="K13" s="175"/>
-      <c r="L13" s="175"/>
-      <c r="M13" s="175"/>
+      <c r="E13" s="190"/>
+      <c r="F13" s="190"/>
+      <c r="G13" s="190"/>
+      <c r="H13" s="190"/>
+      <c r="I13" s="190"/>
+      <c r="J13" s="190"/>
+      <c r="K13" s="190"/>
+      <c r="L13" s="190"/>
+      <c r="M13" s="190"/>
     </row>
     <row r="14" spans="1:13" ht="39.450000000000003" customHeight="1">
-      <c r="A14" s="193"/>
+      <c r="A14" s="208"/>
       <c r="B14" s="2" t="s">
         <v>19</v>
       </c>
       <c r="C14" s="153" t="s">
         <v>11</v>
       </c>
-      <c r="D14" s="176" t="s">
+      <c r="D14" s="191" t="s">
         <v>20</v>
       </c>
-      <c r="E14" s="176"/>
-      <c r="F14" s="176"/>
-      <c r="G14" s="176"/>
-      <c r="H14" s="176"/>
-      <c r="I14" s="176"/>
-      <c r="J14" s="176"/>
-      <c r="K14" s="176"/>
-      <c r="L14" s="176"/>
-      <c r="M14" s="176"/>
+      <c r="E14" s="191"/>
+      <c r="F14" s="191"/>
+      <c r="G14" s="191"/>
+      <c r="H14" s="191"/>
+      <c r="I14" s="191"/>
+      <c r="J14" s="191"/>
+      <c r="K14" s="191"/>
+      <c r="L14" s="191"/>
+      <c r="M14" s="191"/>
     </row>
     <row r="15" spans="1:13" ht="62.7" customHeight="1">
-      <c r="A15" s="193"/>
+      <c r="A15" s="208"/>
       <c r="B15" s="10" t="s">
         <v>21</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="D15" s="201" t="s">
+      <c r="D15" s="216" t="s">
         <v>23</v>
       </c>
-      <c r="E15" s="202"/>
-      <c r="F15" s="202"/>
-      <c r="G15" s="202"/>
-      <c r="H15" s="202"/>
-      <c r="I15" s="202"/>
-      <c r="J15" s="202"/>
-      <c r="K15" s="202"/>
-      <c r="L15" s="202"/>
-      <c r="M15" s="202"/>
+      <c r="E15" s="217"/>
+      <c r="F15" s="217"/>
+      <c r="G15" s="217"/>
+      <c r="H15" s="217"/>
+      <c r="I15" s="217"/>
+      <c r="J15" s="217"/>
+      <c r="K15" s="217"/>
+      <c r="L15" s="217"/>
+      <c r="M15" s="217"/>
     </row>
     <row r="16" spans="1:13" ht="28.95" customHeight="1">
-      <c r="A16" s="190" t="s">
+      <c r="A16" s="205" t="s">
         <v>24</v>
       </c>
       <c r="B16" s="3" t="s">
@@ -4203,357 +4161,357 @@
       <c r="C16" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="D16" s="177" t="s">
+      <c r="D16" s="192" t="s">
         <v>26</v>
       </c>
-      <c r="E16" s="177"/>
-      <c r="F16" s="177"/>
-      <c r="G16" s="177"/>
-      <c r="H16" s="177"/>
-      <c r="I16" s="177"/>
-      <c r="J16" s="177"/>
-      <c r="K16" s="177"/>
-      <c r="L16" s="177"/>
-      <c r="M16" s="177"/>
+      <c r="E16" s="192"/>
+      <c r="F16" s="192"/>
+      <c r="G16" s="192"/>
+      <c r="H16" s="192"/>
+      <c r="I16" s="192"/>
+      <c r="J16" s="192"/>
+      <c r="K16" s="192"/>
+      <c r="L16" s="192"/>
+      <c r="M16" s="192"/>
     </row>
     <row r="17" spans="1:13" ht="43.2">
-      <c r="A17" s="190"/>
+      <c r="A17" s="205"/>
       <c r="B17" s="3" t="s">
         <v>27</v>
       </c>
       <c r="C17" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="D17" s="177" t="s">
+      <c r="D17" s="192" t="s">
         <v>28</v>
       </c>
-      <c r="E17" s="177"/>
-      <c r="F17" s="177"/>
-      <c r="G17" s="177"/>
-      <c r="H17" s="177"/>
-      <c r="I17" s="177"/>
-      <c r="J17" s="177"/>
-      <c r="K17" s="177"/>
-      <c r="L17" s="177"/>
-      <c r="M17" s="177"/>
+      <c r="E17" s="192"/>
+      <c r="F17" s="192"/>
+      <c r="G17" s="192"/>
+      <c r="H17" s="192"/>
+      <c r="I17" s="192"/>
+      <c r="J17" s="192"/>
+      <c r="K17" s="192"/>
+      <c r="L17" s="192"/>
+      <c r="M17" s="192"/>
     </row>
     <row r="18" spans="1:13" ht="28.95" customHeight="1">
-      <c r="A18" s="190"/>
+      <c r="A18" s="205"/>
       <c r="B18" s="3" t="s">
         <v>29</v>
       </c>
       <c r="C18" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="D18" s="181" t="s">
+      <c r="D18" s="196" t="s">
         <v>30</v>
       </c>
-      <c r="E18" s="181"/>
-      <c r="F18" s="181"/>
-      <c r="G18" s="181"/>
-      <c r="H18" s="181"/>
-      <c r="I18" s="181"/>
-      <c r="J18" s="181"/>
-      <c r="K18" s="181"/>
-      <c r="L18" s="181"/>
-      <c r="M18" s="181"/>
+      <c r="E18" s="196"/>
+      <c r="F18" s="196"/>
+      <c r="G18" s="196"/>
+      <c r="H18" s="196"/>
+      <c r="I18" s="196"/>
+      <c r="J18" s="196"/>
+      <c r="K18" s="196"/>
+      <c r="L18" s="196"/>
+      <c r="M18" s="196"/>
     </row>
     <row r="19" spans="1:13" ht="28.8">
-      <c r="A19" s="190"/>
+      <c r="A19" s="205"/>
       <c r="B19" s="3" t="s">
         <v>31</v>
       </c>
       <c r="C19" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="D19" s="177" t="s">
+      <c r="D19" s="192" t="s">
         <v>32</v>
       </c>
-      <c r="E19" s="177"/>
-      <c r="F19" s="177"/>
-      <c r="G19" s="177"/>
-      <c r="H19" s="177"/>
-      <c r="I19" s="177"/>
-      <c r="J19" s="177"/>
-      <c r="K19" s="177"/>
-      <c r="L19" s="177"/>
-      <c r="M19" s="177"/>
+      <c r="E19" s="192"/>
+      <c r="F19" s="192"/>
+      <c r="G19" s="192"/>
+      <c r="H19" s="192"/>
+      <c r="I19" s="192"/>
+      <c r="J19" s="192"/>
+      <c r="K19" s="192"/>
+      <c r="L19" s="192"/>
+      <c r="M19" s="192"/>
     </row>
     <row r="20" spans="1:13" ht="72" customHeight="1">
-      <c r="A20" s="190"/>
+      <c r="A20" s="205"/>
       <c r="B20" s="4" t="s">
         <v>33</v>
       </c>
       <c r="C20" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="D20" s="181" t="s">
+      <c r="D20" s="196" t="s">
         <v>34</v>
       </c>
-      <c r="E20" s="177"/>
-      <c r="F20" s="177"/>
-      <c r="G20" s="177"/>
-      <c r="H20" s="177"/>
-      <c r="I20" s="177"/>
-      <c r="J20" s="177"/>
-      <c r="K20" s="177"/>
-      <c r="L20" s="177"/>
-      <c r="M20" s="177"/>
+      <c r="E20" s="192"/>
+      <c r="F20" s="192"/>
+      <c r="G20" s="192"/>
+      <c r="H20" s="192"/>
+      <c r="I20" s="192"/>
+      <c r="J20" s="192"/>
+      <c r="K20" s="192"/>
+      <c r="L20" s="192"/>
+      <c r="M20" s="192"/>
     </row>
     <row r="21" spans="1:13" ht="24" customHeight="1">
-      <c r="A21" s="190"/>
+      <c r="A21" s="205"/>
       <c r="B21" s="3" t="s">
         <v>35</v>
       </c>
       <c r="C21" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="D21" s="203" t="s">
+      <c r="D21" s="218" t="s">
         <v>36</v>
       </c>
-      <c r="E21" s="179"/>
-      <c r="F21" s="179"/>
-      <c r="G21" s="179"/>
-      <c r="H21" s="179"/>
-      <c r="I21" s="179"/>
-      <c r="J21" s="179"/>
-      <c r="K21" s="179"/>
-      <c r="L21" s="179"/>
-      <c r="M21" s="180"/>
+      <c r="E21" s="194"/>
+      <c r="F21" s="194"/>
+      <c r="G21" s="194"/>
+      <c r="H21" s="194"/>
+      <c r="I21" s="194"/>
+      <c r="J21" s="194"/>
+      <c r="K21" s="194"/>
+      <c r="L21" s="194"/>
+      <c r="M21" s="195"/>
     </row>
     <row r="22" spans="1:13" ht="14.7" customHeight="1">
-      <c r="A22" s="190"/>
+      <c r="A22" s="205"/>
       <c r="B22" s="4" t="s">
         <v>37</v>
       </c>
       <c r="C22" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="D22" s="177" t="s">
+      <c r="D22" s="192" t="s">
         <v>38</v>
       </c>
-      <c r="E22" s="177"/>
-      <c r="F22" s="177"/>
-      <c r="G22" s="177"/>
-      <c r="H22" s="177"/>
-      <c r="I22" s="177"/>
-      <c r="J22" s="177"/>
-      <c r="K22" s="177"/>
-      <c r="L22" s="177"/>
-      <c r="M22" s="177"/>
+      <c r="E22" s="192"/>
+      <c r="F22" s="192"/>
+      <c r="G22" s="192"/>
+      <c r="H22" s="192"/>
+      <c r="I22" s="192"/>
+      <c r="J22" s="192"/>
+      <c r="K22" s="192"/>
+      <c r="L22" s="192"/>
+      <c r="M22" s="192"/>
     </row>
     <row r="23" spans="1:13" ht="43.2">
-      <c r="A23" s="190"/>
+      <c r="A23" s="205"/>
       <c r="B23" s="3" t="s">
         <v>39</v>
       </c>
       <c r="C23" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="D23" s="177" t="s">
+      <c r="D23" s="192" t="s">
         <v>40</v>
       </c>
-      <c r="E23" s="177"/>
-      <c r="F23" s="177"/>
-      <c r="G23" s="177"/>
-      <c r="H23" s="177"/>
-      <c r="I23" s="177"/>
-      <c r="J23" s="177"/>
-      <c r="K23" s="177"/>
-      <c r="L23" s="177"/>
-      <c r="M23" s="177"/>
+      <c r="E23" s="192"/>
+      <c r="F23" s="192"/>
+      <c r="G23" s="192"/>
+      <c r="H23" s="192"/>
+      <c r="I23" s="192"/>
+      <c r="J23" s="192"/>
+      <c r="K23" s="192"/>
+      <c r="L23" s="192"/>
+      <c r="M23" s="192"/>
     </row>
     <row r="24" spans="1:13" ht="43.2">
-      <c r="A24" s="190"/>
+      <c r="A24" s="205"/>
       <c r="B24" s="3" t="s">
         <v>41</v>
       </c>
       <c r="C24" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="D24" s="181" t="s">
+      <c r="D24" s="196" t="s">
         <v>42</v>
       </c>
-      <c r="E24" s="181"/>
-      <c r="F24" s="181"/>
-      <c r="G24" s="181"/>
-      <c r="H24" s="181"/>
-      <c r="I24" s="181"/>
-      <c r="J24" s="181"/>
-      <c r="K24" s="181"/>
-      <c r="L24" s="181"/>
-      <c r="M24" s="181"/>
+      <c r="E24" s="196"/>
+      <c r="F24" s="196"/>
+      <c r="G24" s="196"/>
+      <c r="H24" s="196"/>
+      <c r="I24" s="196"/>
+      <c r="J24" s="196"/>
+      <c r="K24" s="196"/>
+      <c r="L24" s="196"/>
+      <c r="M24" s="196"/>
     </row>
     <row r="25" spans="1:13">
-      <c r="A25" s="190"/>
+      <c r="A25" s="205"/>
       <c r="B25" s="3" t="s">
         <v>43</v>
       </c>
       <c r="C25" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="D25" s="177" t="s">
+      <c r="D25" s="192" t="s">
         <v>44</v>
       </c>
-      <c r="E25" s="177"/>
-      <c r="F25" s="177"/>
-      <c r="G25" s="177"/>
-      <c r="H25" s="177"/>
-      <c r="I25" s="177"/>
-      <c r="J25" s="177"/>
-      <c r="K25" s="177"/>
-      <c r="L25" s="177"/>
-      <c r="M25" s="177"/>
+      <c r="E25" s="192"/>
+      <c r="F25" s="192"/>
+      <c r="G25" s="192"/>
+      <c r="H25" s="192"/>
+      <c r="I25" s="192"/>
+      <c r="J25" s="192"/>
+      <c r="K25" s="192"/>
+      <c r="L25" s="192"/>
+      <c r="M25" s="192"/>
     </row>
     <row r="26" spans="1:13" ht="28.8">
-      <c r="A26" s="190"/>
+      <c r="A26" s="205"/>
       <c r="B26" s="3" t="s">
         <v>45</v>
       </c>
       <c r="C26" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="D26" s="177" t="s">
+      <c r="D26" s="192" t="s">
         <v>46</v>
       </c>
-      <c r="E26" s="177"/>
-      <c r="F26" s="177"/>
-      <c r="G26" s="177"/>
-      <c r="H26" s="177"/>
-      <c r="I26" s="177"/>
-      <c r="J26" s="177"/>
-      <c r="K26" s="177"/>
-      <c r="L26" s="177"/>
-      <c r="M26" s="177"/>
+      <c r="E26" s="192"/>
+      <c r="F26" s="192"/>
+      <c r="G26" s="192"/>
+      <c r="H26" s="192"/>
+      <c r="I26" s="192"/>
+      <c r="J26" s="192"/>
+      <c r="K26" s="192"/>
+      <c r="L26" s="192"/>
+      <c r="M26" s="192"/>
     </row>
     <row r="27" spans="1:13">
-      <c r="A27" s="190"/>
+      <c r="A27" s="205"/>
       <c r="B27" s="3" t="s">
         <v>47</v>
       </c>
       <c r="C27" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="D27" s="177" t="s">
+      <c r="D27" s="192" t="s">
         <v>48</v>
       </c>
-      <c r="E27" s="177"/>
-      <c r="F27" s="177"/>
-      <c r="G27" s="177"/>
-      <c r="H27" s="177"/>
-      <c r="I27" s="177"/>
-      <c r="J27" s="177"/>
-      <c r="K27" s="177"/>
-      <c r="L27" s="177"/>
-      <c r="M27" s="177"/>
+      <c r="E27" s="192"/>
+      <c r="F27" s="192"/>
+      <c r="G27" s="192"/>
+      <c r="H27" s="192"/>
+      <c r="I27" s="192"/>
+      <c r="J27" s="192"/>
+      <c r="K27" s="192"/>
+      <c r="L27" s="192"/>
+      <c r="M27" s="192"/>
     </row>
     <row r="28" spans="1:13">
-      <c r="A28" s="190"/>
+      <c r="A28" s="205"/>
       <c r="B28" s="4" t="s">
         <v>49</v>
       </c>
       <c r="C28" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="D28" s="177" t="s">
+      <c r="D28" s="192" t="s">
         <v>50</v>
       </c>
-      <c r="E28" s="177"/>
-      <c r="F28" s="177"/>
-      <c r="G28" s="177"/>
-      <c r="H28" s="177"/>
-      <c r="I28" s="177"/>
-      <c r="J28" s="177"/>
-      <c r="K28" s="177"/>
-      <c r="L28" s="177"/>
-      <c r="M28" s="177"/>
+      <c r="E28" s="192"/>
+      <c r="F28" s="192"/>
+      <c r="G28" s="192"/>
+      <c r="H28" s="192"/>
+      <c r="I28" s="192"/>
+      <c r="J28" s="192"/>
+      <c r="K28" s="192"/>
+      <c r="L28" s="192"/>
+      <c r="M28" s="192"/>
     </row>
     <row r="29" spans="1:13" ht="33" customHeight="1">
-      <c r="A29" s="190"/>
+      <c r="A29" s="205"/>
       <c r="B29" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C29" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="D29" s="178" t="s">
+      <c r="D29" s="193" t="s">
         <v>52</v>
       </c>
-      <c r="E29" s="179"/>
-      <c r="F29" s="179"/>
-      <c r="G29" s="179"/>
-      <c r="H29" s="179"/>
-      <c r="I29" s="179"/>
-      <c r="J29" s="179"/>
-      <c r="K29" s="179"/>
-      <c r="L29" s="179"/>
-      <c r="M29" s="180"/>
+      <c r="E29" s="194"/>
+      <c r="F29" s="194"/>
+      <c r="G29" s="194"/>
+      <c r="H29" s="194"/>
+      <c r="I29" s="194"/>
+      <c r="J29" s="194"/>
+      <c r="K29" s="194"/>
+      <c r="L29" s="194"/>
+      <c r="M29" s="195"/>
     </row>
     <row r="30" spans="1:13">
-      <c r="A30" s="190"/>
+      <c r="A30" s="205"/>
       <c r="B30" s="3" t="s">
         <v>53</v>
       </c>
       <c r="C30" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="D30" s="177" t="s">
+      <c r="D30" s="192" t="s">
         <v>54</v>
       </c>
-      <c r="E30" s="177"/>
-      <c r="F30" s="177"/>
-      <c r="G30" s="177"/>
-      <c r="H30" s="177"/>
-      <c r="I30" s="177"/>
-      <c r="J30" s="177"/>
-      <c r="K30" s="177"/>
-      <c r="L30" s="177"/>
-      <c r="M30" s="177"/>
+      <c r="E30" s="192"/>
+      <c r="F30" s="192"/>
+      <c r="G30" s="192"/>
+      <c r="H30" s="192"/>
+      <c r="I30" s="192"/>
+      <c r="J30" s="192"/>
+      <c r="K30" s="192"/>
+      <c r="L30" s="192"/>
+      <c r="M30" s="192"/>
     </row>
     <row r="31" spans="1:13">
-      <c r="A31" s="190"/>
+      <c r="A31" s="205"/>
       <c r="B31" s="3" t="s">
         <v>55</v>
       </c>
       <c r="C31" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="D31" s="177" t="s">
+      <c r="D31" s="192" t="s">
         <v>56</v>
       </c>
-      <c r="E31" s="177"/>
-      <c r="F31" s="177"/>
-      <c r="G31" s="177"/>
-      <c r="H31" s="177"/>
-      <c r="I31" s="177"/>
-      <c r="J31" s="177"/>
-      <c r="K31" s="177"/>
-      <c r="L31" s="177"/>
-      <c r="M31" s="177"/>
+      <c r="E31" s="192"/>
+      <c r="F31" s="192"/>
+      <c r="G31" s="192"/>
+      <c r="H31" s="192"/>
+      <c r="I31" s="192"/>
+      <c r="J31" s="192"/>
+      <c r="K31" s="192"/>
+      <c r="L31" s="192"/>
+      <c r="M31" s="192"/>
     </row>
     <row r="32" spans="1:13">
-      <c r="A32" s="190"/>
+      <c r="A32" s="205"/>
       <c r="B32" s="4" t="s">
         <v>57</v>
       </c>
       <c r="C32" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="D32" s="177" t="s">
+      <c r="D32" s="192" t="s">
         <v>58</v>
       </c>
-      <c r="E32" s="177"/>
-      <c r="F32" s="177"/>
-      <c r="G32" s="177"/>
-      <c r="H32" s="177"/>
-      <c r="I32" s="177"/>
-      <c r="J32" s="177"/>
-      <c r="K32" s="177"/>
-      <c r="L32" s="177"/>
-      <c r="M32" s="177"/>
+      <c r="E32" s="192"/>
+      <c r="F32" s="192"/>
+      <c r="G32" s="192"/>
+      <c r="H32" s="192"/>
+      <c r="I32" s="192"/>
+      <c r="J32" s="192"/>
+      <c r="K32" s="192"/>
+      <c r="L32" s="192"/>
+      <c r="M32" s="192"/>
     </row>
     <row r="33" spans="1:13">
-      <c r="A33" s="191" t="s">
+      <c r="A33" s="206" t="s">
         <v>59</v>
       </c>
       <c r="B33" s="5" t="s">
@@ -4562,249 +4520,249 @@
       <c r="C33" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="D33" s="185" t="s">
+      <c r="D33" s="200" t="s">
         <v>61</v>
       </c>
-      <c r="E33" s="185"/>
-      <c r="F33" s="185"/>
-      <c r="G33" s="185"/>
-      <c r="H33" s="185"/>
-      <c r="I33" s="185"/>
-      <c r="J33" s="185"/>
-      <c r="K33" s="185"/>
-      <c r="L33" s="185"/>
-      <c r="M33" s="185"/>
+      <c r="E33" s="200"/>
+      <c r="F33" s="200"/>
+      <c r="G33" s="200"/>
+      <c r="H33" s="200"/>
+      <c r="I33" s="200"/>
+      <c r="J33" s="200"/>
+      <c r="K33" s="200"/>
+      <c r="L33" s="200"/>
+      <c r="M33" s="200"/>
     </row>
     <row r="34" spans="1:13" ht="79.2" customHeight="1">
-      <c r="A34" s="191"/>
+      <c r="A34" s="206"/>
       <c r="B34" s="6" t="s">
         <v>33</v>
       </c>
       <c r="C34" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="D34" s="186" t="s">
+      <c r="D34" s="201" t="s">
         <v>34</v>
       </c>
-      <c r="E34" s="185"/>
-      <c r="F34" s="185"/>
-      <c r="G34" s="185"/>
-      <c r="H34" s="185"/>
-      <c r="I34" s="185"/>
-      <c r="J34" s="185"/>
-      <c r="K34" s="185"/>
-      <c r="L34" s="185"/>
-      <c r="M34" s="185"/>
+      <c r="E34" s="200"/>
+      <c r="F34" s="200"/>
+      <c r="G34" s="200"/>
+      <c r="H34" s="200"/>
+      <c r="I34" s="200"/>
+      <c r="J34" s="200"/>
+      <c r="K34" s="200"/>
+      <c r="L34" s="200"/>
+      <c r="M34" s="200"/>
     </row>
     <row r="35" spans="1:13" ht="28.8">
-      <c r="A35" s="191"/>
+      <c r="A35" s="206"/>
       <c r="B35" s="5" t="s">
         <v>62</v>
       </c>
       <c r="C35" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="D35" s="182" t="s">
+      <c r="D35" s="197" t="s">
         <v>36</v>
       </c>
-      <c r="E35" s="183"/>
-      <c r="F35" s="183"/>
-      <c r="G35" s="183"/>
-      <c r="H35" s="183"/>
-      <c r="I35" s="183"/>
-      <c r="J35" s="183"/>
-      <c r="K35" s="183"/>
-      <c r="L35" s="183"/>
-      <c r="M35" s="184"/>
+      <c r="E35" s="198"/>
+      <c r="F35" s="198"/>
+      <c r="G35" s="198"/>
+      <c r="H35" s="198"/>
+      <c r="I35" s="198"/>
+      <c r="J35" s="198"/>
+      <c r="K35" s="198"/>
+      <c r="L35" s="198"/>
+      <c r="M35" s="199"/>
     </row>
     <row r="36" spans="1:13">
-      <c r="A36" s="191"/>
+      <c r="A36" s="206"/>
       <c r="B36" s="6" t="s">
         <v>37</v>
       </c>
       <c r="C36" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="D36" s="185" t="s">
+      <c r="D36" s="200" t="s">
         <v>38</v>
       </c>
-      <c r="E36" s="185"/>
-      <c r="F36" s="185"/>
-      <c r="G36" s="185"/>
-      <c r="H36" s="185"/>
-      <c r="I36" s="185"/>
-      <c r="J36" s="185"/>
-      <c r="K36" s="185"/>
-      <c r="L36" s="185"/>
-      <c r="M36" s="185"/>
+      <c r="E36" s="200"/>
+      <c r="F36" s="200"/>
+      <c r="G36" s="200"/>
+      <c r="H36" s="200"/>
+      <c r="I36" s="200"/>
+      <c r="J36" s="200"/>
+      <c r="K36" s="200"/>
+      <c r="L36" s="200"/>
+      <c r="M36" s="200"/>
     </row>
     <row r="37" spans="1:13" ht="43.2">
-      <c r="A37" s="191"/>
+      <c r="A37" s="206"/>
       <c r="B37" s="5" t="s">
         <v>39</v>
       </c>
       <c r="C37" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="D37" s="185" t="s">
+      <c r="D37" s="200" t="s">
         <v>40</v>
       </c>
-      <c r="E37" s="185"/>
-      <c r="F37" s="185"/>
-      <c r="G37" s="185"/>
-      <c r="H37" s="185"/>
-      <c r="I37" s="185"/>
-      <c r="J37" s="185"/>
-      <c r="K37" s="185"/>
-      <c r="L37" s="185"/>
-      <c r="M37" s="185"/>
+      <c r="E37" s="200"/>
+      <c r="F37" s="200"/>
+      <c r="G37" s="200"/>
+      <c r="H37" s="200"/>
+      <c r="I37" s="200"/>
+      <c r="J37" s="200"/>
+      <c r="K37" s="200"/>
+      <c r="L37" s="200"/>
+      <c r="M37" s="200"/>
     </row>
     <row r="38" spans="1:13">
-      <c r="A38" s="191"/>
+      <c r="A38" s="206"/>
       <c r="B38" s="5" t="s">
         <v>63</v>
       </c>
       <c r="C38" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="D38" s="185" t="s">
+      <c r="D38" s="200" t="s">
         <v>64</v>
       </c>
-      <c r="E38" s="185"/>
-      <c r="F38" s="185"/>
-      <c r="G38" s="185"/>
-      <c r="H38" s="185"/>
-      <c r="I38" s="185"/>
-      <c r="J38" s="185"/>
-      <c r="K38" s="185"/>
-      <c r="L38" s="185"/>
-      <c r="M38" s="185"/>
+      <c r="E38" s="200"/>
+      <c r="F38" s="200"/>
+      <c r="G38" s="200"/>
+      <c r="H38" s="200"/>
+      <c r="I38" s="200"/>
+      <c r="J38" s="200"/>
+      <c r="K38" s="200"/>
+      <c r="L38" s="200"/>
+      <c r="M38" s="200"/>
     </row>
     <row r="39" spans="1:13">
-      <c r="A39" s="191"/>
+      <c r="A39" s="206"/>
       <c r="B39" s="6" t="s">
         <v>65</v>
       </c>
       <c r="C39" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="D39" s="185" t="s">
+      <c r="D39" s="200" t="s">
         <v>44</v>
       </c>
-      <c r="E39" s="185"/>
-      <c r="F39" s="185"/>
-      <c r="G39" s="185"/>
-      <c r="H39" s="185"/>
-      <c r="I39" s="185"/>
-      <c r="J39" s="185"/>
-      <c r="K39" s="185"/>
-      <c r="L39" s="185"/>
-      <c r="M39" s="185"/>
+      <c r="E39" s="200"/>
+      <c r="F39" s="200"/>
+      <c r="G39" s="200"/>
+      <c r="H39" s="200"/>
+      <c r="I39" s="200"/>
+      <c r="J39" s="200"/>
+      <c r="K39" s="200"/>
+      <c r="L39" s="200"/>
+      <c r="M39" s="200"/>
     </row>
     <row r="40" spans="1:13">
-      <c r="A40" s="191"/>
+      <c r="A40" s="206"/>
       <c r="B40" s="6" t="s">
         <v>49</v>
       </c>
       <c r="C40" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="D40" s="185" t="s">
+      <c r="D40" s="200" t="s">
         <v>50</v>
       </c>
-      <c r="E40" s="185"/>
-      <c r="F40" s="185"/>
-      <c r="G40" s="185"/>
-      <c r="H40" s="185"/>
-      <c r="I40" s="185"/>
-      <c r="J40" s="185"/>
-      <c r="K40" s="185"/>
-      <c r="L40" s="185"/>
-      <c r="M40" s="185"/>
+      <c r="E40" s="200"/>
+      <c r="F40" s="200"/>
+      <c r="G40" s="200"/>
+      <c r="H40" s="200"/>
+      <c r="I40" s="200"/>
+      <c r="J40" s="200"/>
+      <c r="K40" s="200"/>
+      <c r="L40" s="200"/>
+      <c r="M40" s="200"/>
     </row>
     <row r="41" spans="1:13" ht="43.2">
-      <c r="A41" s="191"/>
+      <c r="A41" s="206"/>
       <c r="B41" s="5" t="s">
         <v>66</v>
       </c>
       <c r="C41" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="D41" s="198" t="s">
+      <c r="D41" s="213" t="s">
         <v>67</v>
       </c>
-      <c r="E41" s="199"/>
-      <c r="F41" s="199"/>
-      <c r="G41" s="199"/>
-      <c r="H41" s="199"/>
-      <c r="I41" s="199"/>
-      <c r="J41" s="199"/>
-      <c r="K41" s="199"/>
-      <c r="L41" s="199"/>
-      <c r="M41" s="200"/>
+      <c r="E41" s="214"/>
+      <c r="F41" s="214"/>
+      <c r="G41" s="214"/>
+      <c r="H41" s="214"/>
+      <c r="I41" s="214"/>
+      <c r="J41" s="214"/>
+      <c r="K41" s="214"/>
+      <c r="L41" s="214"/>
+      <c r="M41" s="215"/>
     </row>
     <row r="42" spans="1:13">
-      <c r="A42" s="191"/>
+      <c r="A42" s="206"/>
       <c r="B42" s="5" t="s">
         <v>68</v>
       </c>
       <c r="C42" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="D42" s="185" t="s">
+      <c r="D42" s="200" t="s">
         <v>54</v>
       </c>
-      <c r="E42" s="185"/>
-      <c r="F42" s="185"/>
-      <c r="G42" s="185"/>
-      <c r="H42" s="185"/>
-      <c r="I42" s="185"/>
-      <c r="J42" s="185"/>
-      <c r="K42" s="185"/>
-      <c r="L42" s="185"/>
-      <c r="M42" s="185"/>
+      <c r="E42" s="200"/>
+      <c r="F42" s="200"/>
+      <c r="G42" s="200"/>
+      <c r="H42" s="200"/>
+      <c r="I42" s="200"/>
+      <c r="J42" s="200"/>
+      <c r="K42" s="200"/>
+      <c r="L42" s="200"/>
+      <c r="M42" s="200"/>
     </row>
     <row r="43" spans="1:13">
-      <c r="A43" s="191"/>
+      <c r="A43" s="206"/>
       <c r="B43" s="5" t="s">
         <v>69</v>
       </c>
       <c r="C43" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="D43" s="185" t="s">
+      <c r="D43" s="200" t="s">
         <v>56</v>
       </c>
-      <c r="E43" s="185"/>
-      <c r="F43" s="185"/>
-      <c r="G43" s="185"/>
-      <c r="H43" s="185"/>
-      <c r="I43" s="185"/>
-      <c r="J43" s="185"/>
-      <c r="K43" s="185"/>
-      <c r="L43" s="185"/>
-      <c r="M43" s="185"/>
+      <c r="E43" s="200"/>
+      <c r="F43" s="200"/>
+      <c r="G43" s="200"/>
+      <c r="H43" s="200"/>
+      <c r="I43" s="200"/>
+      <c r="J43" s="200"/>
+      <c r="K43" s="200"/>
+      <c r="L43" s="200"/>
+      <c r="M43" s="200"/>
     </row>
     <row r="44" spans="1:13">
-      <c r="A44" s="191"/>
+      <c r="A44" s="206"/>
       <c r="B44" s="6" t="s">
         <v>57</v>
       </c>
       <c r="C44" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="D44" s="185" t="s">
+      <c r="D44" s="200" t="s">
         <v>58</v>
       </c>
-      <c r="E44" s="185"/>
-      <c r="F44" s="185"/>
-      <c r="G44" s="185"/>
-      <c r="H44" s="185"/>
-      <c r="I44" s="185"/>
-      <c r="J44" s="185"/>
-      <c r="K44" s="185"/>
-      <c r="L44" s="185"/>
-      <c r="M44" s="185"/>
+      <c r="E44" s="200"/>
+      <c r="F44" s="200"/>
+      <c r="G44" s="200"/>
+      <c r="H44" s="200"/>
+      <c r="I44" s="200"/>
+      <c r="J44" s="200"/>
+      <c r="K44" s="200"/>
+      <c r="L44" s="200"/>
+      <c r="M44" s="200"/>
     </row>
   </sheetData>
   <mergeCells count="43">
@@ -4888,48 +4846,48 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:34" ht="23.4">
-      <c r="A1" s="173" t="s">
+      <c r="A1" s="223" t="s">
         <v>70</v>
       </c>
-      <c r="B1" s="174"/>
-      <c r="C1" s="174"/>
-      <c r="D1" s="174"/>
-      <c r="E1" s="174"/>
-      <c r="F1" s="171" t="s">
+      <c r="B1" s="224"/>
+      <c r="C1" s="224"/>
+      <c r="D1" s="224"/>
+      <c r="E1" s="224"/>
+      <c r="F1" s="221" t="s">
         <v>71</v>
       </c>
-      <c r="G1" s="171"/>
-      <c r="H1" s="171"/>
-      <c r="I1" s="171"/>
-      <c r="J1" s="171"/>
-      <c r="K1" s="171"/>
-      <c r="L1" s="171"/>
-      <c r="M1" s="171"/>
-      <c r="N1" s="171"/>
-      <c r="O1" s="171"/>
-      <c r="P1" s="171"/>
-      <c r="Q1" s="171"/>
-      <c r="R1" s="171"/>
-      <c r="S1" s="171"/>
-      <c r="T1" s="171"/>
-      <c r="U1" s="171"/>
-      <c r="V1" s="171"/>
-      <c r="W1" s="172" t="s">
+      <c r="G1" s="221"/>
+      <c r="H1" s="221"/>
+      <c r="I1" s="221"/>
+      <c r="J1" s="221"/>
+      <c r="K1" s="221"/>
+      <c r="L1" s="221"/>
+      <c r="M1" s="221"/>
+      <c r="N1" s="221"/>
+      <c r="O1" s="221"/>
+      <c r="P1" s="221"/>
+      <c r="Q1" s="221"/>
+      <c r="R1" s="221"/>
+      <c r="S1" s="221"/>
+      <c r="T1" s="221"/>
+      <c r="U1" s="221"/>
+      <c r="V1" s="221"/>
+      <c r="W1" s="222" t="s">
         <v>72</v>
       </c>
-      <c r="X1" s="172"/>
-      <c r="Y1" s="172"/>
-      <c r="Z1" s="172"/>
-      <c r="AA1" s="172"/>
-      <c r="AB1" s="172"/>
-      <c r="AC1" s="172"/>
-      <c r="AD1" s="172"/>
-      <c r="AE1" s="172"/>
-      <c r="AF1" s="172"/>
-      <c r="AG1" s="172"/>
-      <c r="AH1" s="172"/>
+      <c r="X1" s="222"/>
+      <c r="Y1" s="222"/>
+      <c r="Z1" s="222"/>
+      <c r="AA1" s="222"/>
+      <c r="AB1" s="222"/>
+      <c r="AC1" s="222"/>
+      <c r="AD1" s="222"/>
+      <c r="AE1" s="222"/>
+      <c r="AF1" s="222"/>
+      <c r="AG1" s="222"/>
+      <c r="AH1" s="222"/>
     </row>
-    <row r="2" spans="1:34" s="65" customFormat="1" ht="103.95" customHeight="1">
+    <row r="2" spans="1:34" s="65" customFormat="1" ht="100.8">
       <c r="A2" s="33" t="s">
         <v>73</v>
       </c>
@@ -5033,7 +4991,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:34" ht="72" hidden="1">
+    <row r="3" spans="1:34" ht="72">
       <c r="A3" s="99" t="s">
         <v>90</v>
       </c>
@@ -5129,7 +5087,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="4" spans="1:34" ht="181.5" hidden="1" customHeight="1">
+    <row r="4" spans="1:34" ht="144">
       <c r="A4" s="99" t="s">
         <v>106</v>
       </c>
@@ -5227,7 +5185,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="5" spans="1:34" hidden="1">
+    <row r="5" spans="1:34">
       <c r="A5" s="24" t="s">
         <v>120</v>
       </c>
@@ -5289,7 +5247,7 @@
       <c r="AG5" s="49"/>
       <c r="AH5" s="49"/>
     </row>
-    <row r="6" spans="1:34" ht="153.44999999999999" customHeight="1">
+    <row r="6" spans="1:34" ht="158.4">
       <c r="A6" s="99" t="s">
         <v>123</v>
       </c>
@@ -5299,101 +5257,101 @@
       <c r="C6" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="D6" s="206" t="s">
+      <c r="D6" s="171" t="s">
         <v>528</v>
       </c>
       <c r="E6" s="59" t="s">
         <v>105</v>
       </c>
-      <c r="F6" s="207" t="s">
+      <c r="F6" s="172" t="s">
         <v>529</v>
       </c>
-      <c r="G6" s="208" t="s">
+      <c r="G6" s="173" t="s">
         <v>121</v>
       </c>
-      <c r="H6" s="207" t="s">
+      <c r="H6" s="172" t="s">
         <v>530</v>
       </c>
-      <c r="I6" s="208" t="s">
+      <c r="I6" s="173" t="s">
         <v>121</v>
       </c>
-      <c r="J6" s="209" t="s">
+      <c r="J6" s="174" t="s">
         <v>96</v>
       </c>
-      <c r="K6" s="210">
+      <c r="K6" s="175">
         <v>45992</v>
       </c>
-      <c r="L6" s="211" t="s">
+      <c r="L6" s="176" t="s">
         <v>531</v>
       </c>
-      <c r="M6" s="209" t="s">
+      <c r="M6" s="174" t="s">
         <v>111</v>
       </c>
-      <c r="N6" s="212" t="s">
-        <v>93</v>
-      </c>
-      <c r="O6" s="213" t="s">
+      <c r="N6" s="177" t="s">
+        <v>93</v>
+      </c>
+      <c r="O6" s="178" t="s">
         <v>532</v>
       </c>
-      <c r="P6" s="214" t="s">
+      <c r="P6" s="179" t="s">
         <v>533</v>
       </c>
-      <c r="Q6" s="213" t="s">
+      <c r="Q6" s="178" t="s">
         <v>534</v>
       </c>
-      <c r="R6" s="215" t="s">
+      <c r="R6" s="180" t="s">
         <v>535</v>
       </c>
-      <c r="S6" s="209" t="s">
-        <v>93</v>
-      </c>
-      <c r="T6" s="207" t="s">
+      <c r="S6" s="174" t="s">
+        <v>93</v>
+      </c>
+      <c r="T6" s="172" t="s">
         <v>529</v>
       </c>
-      <c r="U6" s="207" t="s">
+      <c r="U6" s="172" t="s">
         <v>198</v>
       </c>
-      <c r="V6" s="207" t="s">
+      <c r="V6" s="172" t="s">
         <v>256</v>
       </c>
-      <c r="W6" s="222" t="s">
+      <c r="W6" s="187" t="s">
         <v>548</v>
       </c>
-      <c r="X6" s="216" t="s">
+      <c r="X6" s="181" t="s">
         <v>96</v>
       </c>
-      <c r="Y6" s="216">
+      <c r="Y6" s="181">
         <v>45992</v>
       </c>
-      <c r="Z6" s="221" t="s">
+      <c r="Z6" s="186" t="s">
         <v>547</v>
       </c>
-      <c r="AA6" s="217" t="s">
+      <c r="AA6" s="182" t="s">
         <v>111</v>
       </c>
-      <c r="AB6" s="217" t="s">
-        <v>93</v>
-      </c>
-      <c r="AC6" s="218" t="s">
+      <c r="AB6" s="182" t="s">
+        <v>93</v>
+      </c>
+      <c r="AC6" s="183" t="s">
         <v>532</v>
       </c>
-      <c r="AD6" s="219" t="s">
+      <c r="AD6" s="184" t="s">
         <v>549</v>
       </c>
-      <c r="AE6" s="217" t="s">
-        <v>93</v>
-      </c>
-      <c r="AF6" s="219" t="s">
+      <c r="AE6" s="182" t="s">
+        <v>93</v>
+      </c>
+      <c r="AF6" s="184" t="s">
         <v>529</v>
       </c>
-      <c r="AG6" s="220" t="s">
+      <c r="AG6" s="185" t="s">
         <v>537</v>
       </c>
-      <c r="AH6" s="219" t="s">
+      <c r="AH6" s="184" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="7" spans="1:34" ht="144" hidden="1">
+    <row r="7" spans="1:34" ht="144">
       <c r="A7" s="24" t="s">
         <v>125</v>
       </c>
@@ -5497,7 +5455,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="8" spans="1:34" ht="73.95" hidden="1" customHeight="1">
+    <row r="8" spans="1:34" ht="129.6">
       <c r="A8" s="24" t="s">
         <v>135</v>
       </c>
@@ -5595,7 +5553,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="9" spans="1:34" ht="43.2" hidden="1">
+    <row r="9" spans="1:34" ht="43.2">
       <c r="A9" s="100" t="s">
         <v>148</v>
       </c>
@@ -5689,7 +5647,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="10" spans="1:34" ht="103.95" hidden="1" customHeight="1">
+    <row r="10" spans="1:34">
       <c r="A10" s="24" t="s">
         <v>161</v>
       </c>
@@ -5765,7 +5723,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="11" spans="1:34" ht="120.75" hidden="1" customHeight="1">
+    <row r="11" spans="1:34" ht="158.4">
       <c r="A11" s="99" t="s">
         <v>167</v>
       </c>
@@ -5863,7 +5821,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="12" spans="1:34" ht="100.2" hidden="1" customHeight="1">
+    <row r="12" spans="1:34" ht="216">
       <c r="A12" s="24" t="s">
         <v>173</v>
       </c>
@@ -5963,7 +5921,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="13" spans="1:34" ht="232.2" hidden="1" customHeight="1">
+    <row r="13" spans="1:34" ht="216">
       <c r="A13" s="99" t="s">
         <v>183</v>
       </c>
@@ -6061,7 +6019,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="14" spans="1:34" ht="42.45" hidden="1" customHeight="1">
+    <row r="14" spans="1:34">
       <c r="A14" s="24" t="s">
         <v>189</v>
       </c>
@@ -6109,7 +6067,7 @@
       <c r="AG14" s="42"/>
       <c r="AH14" s="42"/>
     </row>
-    <row r="15" spans="1:34" ht="43.2" hidden="1">
+    <row r="15" spans="1:34" ht="43.2">
       <c r="A15" s="100" t="s">
         <v>190</v>
       </c>
@@ -6213,7 +6171,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="16" spans="1:34" hidden="1">
+    <row r="16" spans="1:34">
       <c r="A16" s="24" t="s">
         <v>203</v>
       </c>
@@ -6259,7 +6217,7 @@
       <c r="AG16" s="42"/>
       <c r="AH16" s="42"/>
     </row>
-    <row r="17" spans="1:34" hidden="1">
+    <row r="17" spans="1:34">
       <c r="A17" s="100" t="s">
         <v>204</v>
       </c>
@@ -6333,12 +6291,12 @@
       <c r="AG17" s="49"/>
       <c r="AH17" s="49"/>
     </row>
-    <row r="18" spans="1:34" ht="158.4" hidden="1">
+    <row r="18" spans="1:34" ht="158.4">
       <c r="A18" s="99" t="s">
         <v>205</v>
       </c>
       <c r="B18" s="18">
-        <v>45999</v>
+        <v>46087</v>
       </c>
       <c r="C18" s="19"/>
       <c r="D18" s="54" t="s">
@@ -6413,7 +6371,7 @@
       <c r="AG18" s="71"/>
       <c r="AH18" s="32"/>
     </row>
-    <row r="19" spans="1:34" ht="181.95" hidden="1" customHeight="1">
+    <row r="19" spans="1:34" ht="158.4">
       <c r="A19" s="24" t="s">
         <v>210</v>
       </c>
@@ -6513,7 +6471,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="20" spans="1:34" ht="158.4" hidden="1">
+    <row r="20" spans="1:34" ht="158.4">
       <c r="A20" s="99" t="s">
         <v>222</v>
       </c>
@@ -6613,7 +6571,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="21" spans="1:34" ht="105" hidden="1" customHeight="1">
+    <row r="21" spans="1:34" ht="158.4">
       <c r="A21" s="99" t="s">
         <v>230</v>
       </c>
@@ -6713,7 +6671,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="22" spans="1:34" ht="219.45" hidden="1" customHeight="1">
+    <row r="22" spans="1:34" ht="388.8">
       <c r="A22" s="99" t="s">
         <v>240</v>
       </c>
@@ -6811,7 +6769,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="23" spans="1:34" ht="85.2" hidden="1" customHeight="1">
+    <row r="23" spans="1:34" ht="100.8">
       <c r="A23" s="24" t="s">
         <v>249</v>
       </c>
@@ -6903,7 +6861,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="24" spans="1:34" ht="124.2" hidden="1" customHeight="1">
+    <row r="24" spans="1:34" ht="158.4">
       <c r="A24" s="99" t="s">
         <v>261</v>
       </c>
@@ -7001,7 +6959,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="25" spans="1:34" ht="110.7" hidden="1" customHeight="1">
+    <row r="25" spans="1:34" ht="316.8">
       <c r="A25" s="99" t="s">
         <v>269</v>
       </c>
@@ -7103,7 +7061,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="26" spans="1:34" ht="65.7" hidden="1" customHeight="1">
+    <row r="26" spans="1:34" ht="57.6">
       <c r="A26" s="24" t="s">
         <v>284</v>
       </c>
@@ -7203,7 +7161,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="27" spans="1:34" hidden="1">
+    <row r="27" spans="1:34">
       <c r="A27" s="24" t="s">
         <v>287</v>
       </c>
@@ -7245,7 +7203,7 @@
       <c r="AG27" s="42"/>
       <c r="AH27" s="42"/>
     </row>
-    <row r="28" spans="1:34" ht="66.45" hidden="1" customHeight="1">
+    <row r="28" spans="1:34" ht="86.4">
       <c r="A28" s="99" t="s">
         <v>288</v>
       </c>
@@ -7345,7 +7303,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="29" spans="1:34" ht="28.8" hidden="1">
+    <row r="29" spans="1:34" ht="28.8">
       <c r="A29" s="24" t="s">
         <v>304</v>
       </c>
@@ -7437,7 +7395,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="30" spans="1:34" ht="97.95" hidden="1" customHeight="1">
+    <row r="30" spans="1:34" ht="115.2">
       <c r="A30" s="99" t="s">
         <v>309</v>
       </c>
@@ -7533,7 +7491,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="31" spans="1:34" s="66" customFormat="1" ht="158.4" hidden="1">
+    <row r="31" spans="1:34" s="66" customFormat="1" ht="158.4">
       <c r="A31" s="101" t="s">
         <v>323</v>
       </c>
@@ -7637,7 +7595,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="32" spans="1:34" s="67" customFormat="1" ht="28.8" hidden="1">
+    <row r="32" spans="1:34" s="67" customFormat="1" ht="28.8">
       <c r="A32" s="102" t="s">
         <v>331</v>
       </c>
@@ -7717,7 +7675,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="33" spans="1:34" ht="207" hidden="1" customHeight="1">
+    <row r="33" spans="1:34" ht="316.8">
       <c r="A33" s="99" t="s">
         <v>337</v>
       </c>
@@ -7817,7 +7775,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="34" spans="1:34" hidden="1">
+    <row r="34" spans="1:34">
       <c r="A34" s="24" t="s">
         <v>349</v>
       </c>
@@ -7867,7 +7825,7 @@
       <c r="AG34" s="42"/>
       <c r="AH34" s="42"/>
     </row>
-    <row r="35" spans="1:34" ht="129.6" hidden="1">
+    <row r="35" spans="1:34" ht="129.6">
       <c r="A35" s="24" t="s">
         <v>351</v>
       </c>
@@ -7965,7 +7923,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="36" spans="1:34" hidden="1">
+    <row r="36" spans="1:34">
       <c r="A36" s="24" t="s">
         <v>357</v>
       </c>
@@ -8011,7 +7969,7 @@
       <c r="AG36" s="42"/>
       <c r="AH36" s="42"/>
     </row>
-    <row r="37" spans="1:34" ht="57.6" hidden="1">
+    <row r="37" spans="1:34" ht="57.6">
       <c r="A37" s="24" t="s">
         <v>358</v>
       </c>
@@ -8099,7 +8057,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="38" spans="1:34" ht="28.8" hidden="1">
+    <row r="38" spans="1:34" ht="28.8">
       <c r="A38" s="24" t="s">
         <v>368</v>
       </c>
@@ -8151,7 +8109,7 @@
       <c r="AG38" s="42"/>
       <c r="AH38" s="42"/>
     </row>
-    <row r="39" spans="1:34" ht="138" hidden="1" customHeight="1">
+    <row r="39" spans="1:34" ht="158.4">
       <c r="A39" s="24" t="s">
         <v>370</v>
       </c>
@@ -8251,7 +8209,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="40" spans="1:34" ht="129.6" hidden="1">
+    <row r="40" spans="1:34" ht="130.19999999999999" thickBot="1">
       <c r="A40" s="24" t="s">
         <v>380</v>
       </c>
@@ -8347,111 +8305,111 @@
         <v>134</v>
       </c>
     </row>
-    <row r="41" spans="1:34" ht="159" hidden="1" thickBot="1">
+    <row r="41" spans="1:34" ht="159" thickBot="1">
       <c r="A41" s="24" t="s">
         <v>386</v>
       </c>
-      <c r="B41" s="223">
-        <v>45967</v>
-      </c>
-      <c r="C41" s="224" t="s">
+      <c r="B41" s="18">
+        <v>46087</v>
+      </c>
+      <c r="C41" s="19" t="s">
         <v>538</v>
       </c>
-      <c r="D41" s="233" t="s">
+      <c r="D41" s="60" t="s">
         <v>539</v>
       </c>
-      <c r="E41" s="232" t="s">
+      <c r="E41" s="59" t="s">
         <v>105</v>
       </c>
-      <c r="F41" s="228" t="s">
+      <c r="F41" s="44" t="s">
         <v>540</v>
       </c>
-      <c r="G41" s="230" t="s">
+      <c r="G41" s="57" t="s">
         <v>121</v>
       </c>
-      <c r="H41" s="235" t="s">
+      <c r="H41" s="81" t="s">
         <v>541</v>
       </c>
-      <c r="I41" s="230" t="s">
+      <c r="I41" s="57" t="s">
         <v>121</v>
       </c>
-      <c r="J41" s="231" t="s">
+      <c r="J41" s="58" t="s">
         <v>96</v>
       </c>
-      <c r="K41" s="236">
+      <c r="K41" s="83">
         <v>45960</v>
       </c>
-      <c r="L41" s="226" t="s">
+      <c r="L41" s="40" t="s">
         <v>542</v>
       </c>
-      <c r="M41" s="231" t="s">
+      <c r="M41" s="58" t="s">
         <v>111</v>
       </c>
-      <c r="N41" s="231" t="s">
-        <v>93</v>
-      </c>
-      <c r="O41" s="231" t="s">
+      <c r="N41" s="58" t="s">
+        <v>93</v>
+      </c>
+      <c r="O41" s="58" t="s">
         <v>532</v>
       </c>
-      <c r="P41" s="234" t="s">
+      <c r="P41" s="61" t="s">
         <v>543</v>
       </c>
-      <c r="Q41" s="231" t="s">
+      <c r="Q41" s="58" t="s">
         <v>130</v>
       </c>
-      <c r="R41" s="237" t="s">
+      <c r="R41" s="188" t="s">
         <v>387</v>
       </c>
-      <c r="S41" s="231" t="s">
-        <v>93</v>
-      </c>
-      <c r="T41" s="226" t="s">
+      <c r="S41" s="58" t="s">
+        <v>93</v>
+      </c>
+      <c r="T41" s="40" t="s">
         <v>544</v>
       </c>
-      <c r="U41" s="238" t="s">
+      <c r="U41" s="189" t="s">
         <v>545</v>
       </c>
-      <c r="V41" s="238" t="s">
+      <c r="V41" s="189" t="s">
         <v>256</v>
       </c>
-      <c r="W41" s="225" t="s">
+      <c r="W41" s="31" t="s">
         <v>546</v>
       </c>
-      <c r="X41" s="227" t="s">
+      <c r="X41" s="41" t="s">
         <v>96</v>
       </c>
-      <c r="Y41" s="229">
+      <c r="Y41" s="52">
         <v>45960</v>
       </c>
-      <c r="Z41" s="225" t="s">
+      <c r="Z41" s="31" t="s">
         <v>542</v>
       </c>
-      <c r="AA41" s="227" t="s">
+      <c r="AA41" s="41" t="s">
         <v>365</v>
       </c>
-      <c r="AB41" s="227" t="s">
-        <v>93</v>
-      </c>
-      <c r="AC41" s="227" t="s">
+      <c r="AB41" s="41" t="s">
+        <v>93</v>
+      </c>
+      <c r="AC41" s="41" t="s">
         <v>532</v>
       </c>
-      <c r="AD41" s="225" t="s">
+      <c r="AD41" s="31" t="s">
         <v>536</v>
       </c>
-      <c r="AE41" s="227" t="s">
-        <v>93</v>
-      </c>
-      <c r="AF41" s="225" t="s">
+      <c r="AE41" s="41" t="s">
+        <v>93</v>
+      </c>
+      <c r="AF41" s="31" t="s">
         <v>544</v>
       </c>
-      <c r="AG41" s="225" t="s">
+      <c r="AG41" s="31" t="s">
         <v>545</v>
       </c>
-      <c r="AH41" s="225" t="s">
+      <c r="AH41" s="31" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="42" spans="1:34" ht="96.45" hidden="1" customHeight="1">
+    <row r="42" spans="1:34" ht="187.2">
       <c r="A42" s="24" t="s">
         <v>388</v>
       </c>
@@ -8549,7 +8507,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="43" spans="1:34" ht="72" hidden="1">
+    <row r="43" spans="1:34" ht="72">
       <c r="A43" s="99" t="s">
         <v>395</v>
       </c>
@@ -8643,7 +8601,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="44" spans="1:34" ht="86.4" hidden="1">
+    <row r="44" spans="1:34" ht="86.4">
       <c r="A44" s="24" t="s">
         <v>409</v>
       </c>
@@ -8743,7 +8701,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="45" spans="1:34" ht="54" hidden="1" customHeight="1">
+    <row r="45" spans="1:34">
       <c r="A45" s="24" t="s">
         <v>421</v>
       </c>
@@ -8791,7 +8749,7 @@
       <c r="AG45" s="42"/>
       <c r="AH45" s="42"/>
     </row>
-    <row r="46" spans="1:34" ht="144" hidden="1">
+    <row r="46" spans="1:34" ht="144">
       <c r="A46" s="24" t="s">
         <v>422</v>
       </c>
@@ -8891,7 +8849,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="47" spans="1:34" ht="57.6" hidden="1">
+    <row r="47" spans="1:34" ht="57.6">
       <c r="A47" s="24" t="s">
         <v>438</v>
       </c>
@@ -8995,7 +8953,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="48" spans="1:34" ht="115.2" hidden="1">
+    <row r="48" spans="1:34" ht="115.2">
       <c r="A48" s="99" t="s">
         <v>450</v>
       </c>
@@ -9093,7 +9051,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="49" spans="1:34" ht="28.8" hidden="1">
+    <row r="49" spans="1:34" ht="28.8">
       <c r="A49" s="100" t="s">
         <v>459</v>
       </c>
@@ -9157,7 +9115,7 @@
       <c r="AG49" s="49"/>
       <c r="AH49" s="49"/>
     </row>
-    <row r="50" spans="1:34" ht="197.7" hidden="1" customHeight="1">
+    <row r="50" spans="1:34" ht="144">
       <c r="A50" s="99" t="s">
         <v>461</v>
       </c>
@@ -9257,7 +9215,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="51" spans="1:34" ht="158.4" hidden="1">
+    <row r="51" spans="1:34" ht="158.4">
       <c r="A51" s="99" t="s">
         <v>474</v>
       </c>
@@ -9355,7 +9313,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="52" spans="1:34" ht="140.69999999999999" hidden="1" customHeight="1">
+    <row r="52" spans="1:34" ht="158.4">
       <c r="A52" s="24" t="s">
         <v>479</v>
       </c>
@@ -9453,7 +9411,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="53" spans="1:34" ht="100.8" hidden="1">
+    <row r="53" spans="1:34" ht="100.8">
       <c r="A53" s="24" t="s">
         <v>489</v>
       </c>
@@ -9557,7 +9515,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="54" spans="1:34" hidden="1">
+    <row r="54" spans="1:34">
       <c r="A54" s="24" t="s">
         <v>507</v>
       </c>
@@ -9619,7 +9577,7 @@
       <c r="AG54" s="42"/>
       <c r="AH54" s="42"/>
     </row>
-    <row r="55" spans="1:34" ht="43.2" hidden="1">
+    <row r="55" spans="1:34" ht="43.2">
       <c r="A55" s="24" t="s">
         <v>510</v>
       </c>
@@ -9711,7 +9669,7 @@
       <c r="AG55" s="49"/>
       <c r="AH55" s="49"/>
     </row>
-    <row r="56" spans="1:34" hidden="1">
+    <row r="56" spans="1:34">
       <c r="A56" s="24" t="s">
         <v>513</v>
       </c>
@@ -9779,7 +9737,7 @@
       <c r="AG56" s="49"/>
       <c r="AH56" s="49"/>
     </row>
-    <row r="57" spans="1:34" hidden="1">
+    <row r="57" spans="1:34">
       <c r="A57" s="24" t="s">
         <v>516</v>
       </c>
@@ -9825,7 +9783,7 @@
       <c r="AG57" s="42"/>
       <c r="AH57" s="42"/>
     </row>
-    <row r="58" spans="1:34" hidden="1">
+    <row r="58" spans="1:34">
       <c r="A58" s="24" t="s">
         <v>517</v>
       </c>

</xml_diff>